<commit_message>
Security assessment: explicit namespaces in Helm manifests, digest pinning for the Flyway migration image, reviewed scanner exceptions annotated inline (Checkov), access-matrix oracle knows the internal-only reference-data rule, security enhancement pack (guideline, epic, developer handbook)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XrJepX28zgjeqhjmoaT1JD
</commit_message>
<xml_diff>
--- a/docs/security/epics/E15_Security_Hardening_and_Assurance.xlsx
+++ b/docs/security/epics/E15_Security_Hardening_and_Assurance.xlsx
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Policy extractor committed under tools/security with tests; CI workflow with ephemeral Docker Compose stack runs security-verification.js and rbac-matrix.js nightly and on release branches; object-level cases for every module.</t>
+          <t>Policy extractor tools/security/rbac-extract-policy.py with unit tests; CI workflow with ephemeral Docker Compose stack runs security-verification.js and rbac-matrix.js nightly and on release branches; object-level cases for every module.</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -4540,12 +4540,12 @@
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>Commit the static policy extractor (expected access policy from @PreAuthorize, URL rules and BFF workspace gating) under tools/security with tests</t>
+          <t>Unit tests and a reviewed baseline for the policy extractor tools/security/rbac-extract-policy.py (expected access policy from @PreAuthorize, URL rules and BFF workspace gating)</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Extractor reproduces the assessment baseline (762 endpoint entries from 89 controllers); unit tests for SpEL constant resolution</t>
+          <t>Extractor output matches the reviewed baseline (assessment: 762 endpoint entries from 89 controllers); unit tests for SpEL constant resolution and URL rules</t>
         </is>
       </c>
       <c r="G35" s="12" t="n">

</xml_diff>